<commit_message>
EPBDS-16836 Fix small, big and median ranking NaN as the largest number, so small(values, 1) disagreed with min and the median of 3, NaN and 1 was 3
</commit_message>
<xml_diff>
--- a/DEV/org.openl.rules.demo/src/org.openl.rules.demo.examples/Example-4-Reference-Guide/rules/7-Functions/AggregateFunctions.xlsx
+++ b/DEV/org.openl.rules.demo/src/org.openl.rules.demo.examples/Example-4-Reference-Guide/rules/7-Functions/AggregateFunctions.xlsx
@@ -1233,7 +1233,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B2:I104"/>
+  <dimension ref="B2:I110"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2.5" customWidth="1" min="1" max="1"/>
@@ -1252,7 +1252,7 @@
     <row r="4" ht="43.5" customHeight="1">
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Empty values are skipped: avg(5, null) is 5, and a function of only empty values or of an empty array is empty. An element of a primitive array, such as int[], cannot be empty: a blank cell is 0 there, and 0 counts, so the average of 1, 2, 0, 0, 6 is 1.8 while the average of 1, 2, 6 is 3. NaN is not skipped: a NaN value makes min and max NaN, wherever it stands, in an array too.</t>
+          <t>Empty values are skipped: avg(5, null) is 5, and a function of only empty values or of an empty array is empty. An element of a primitive array, such as int[], cannot be empty: a blank cell is 0 there, and 0 counts, so the average of 1, 2, 0, 0, 6 is 1.8 while the average of 1, 2, 6 is 3. NaN is not skipped: a NaN value makes min, max, median, small and big NaN, wherever it stands, in an array too.</t>
         </is>
       </c>
     </row>
@@ -1555,326 +1555,311 @@
     <row r="31">
       <c r="B31" s="6" t="inlineStr">
         <is>
-          <t>SmallSkipsEmpties</t>
+          <t>MedianWithNaN</t>
         </is>
       </c>
       <c r="C31" s="7" t="inlineStr">
         <is>
-          <t>= small(new Integer[] {1, 2, null, null, 6}, 3)</t>
+          <t>= median(new Double[] {3, Double.NaN, 1})</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="B32" s="6" t="inlineStr">
         <is>
+          <t>SmallSkipsEmpties</t>
+        </is>
+      </c>
+      <c r="C32" s="7" t="inlineStr">
+        <is>
+          <t>= small(new Integer[] {1, 2, null, null, 6}, 3)</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="B33" s="6" t="inlineStr">
+        <is>
           <t>SmallWithZeros</t>
         </is>
       </c>
-      <c r="C32" s="7" t="inlineStr">
+      <c r="C33" s="7" t="inlineStr">
         <is>
           <t>= small(new int[] {1, 2, 0, 0, 6}, 3)</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="B34" s="3" t="inlineStr">
+      <c r="B34" s="6" t="inlineStr">
+        <is>
+          <t>SmallWithNaN</t>
+        </is>
+      </c>
+      <c r="C34" s="7" t="inlineStr">
+        <is>
+          <t>= small(new Double[] {3, Double.NaN, 1}, 1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="B35" s="6" t="inlineStr">
+        <is>
+          <t>BigWithNaN</t>
+        </is>
+      </c>
+      <c r="C35" s="7" t="inlineStr">
+        <is>
+          <t>= big(new double[] {3, Double.NaN, 1}, 2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="B37" s="3" t="inlineStr">
         <is>
           <t>Test AggregatesOfEmpty AggregatesOfEmptyTest</t>
         </is>
       </c>
-      <c r="C34" s="8" t="n"/>
-      <c r="D34" s="4" t="n"/>
-    </row>
-    <row r="35">
-      <c r="B35" s="9" t="inlineStr">
-        <is>
-          <t>_res_.$AvgWithEmpty</t>
-        </is>
-      </c>
-      <c r="C35" s="5" t="inlineStr">
-        <is>
-          <t>avg(5, null)</t>
-        </is>
-      </c>
-      <c r="D35" s="10" t="n">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="36">
-      <c r="B36" s="9" t="inlineStr">
-        <is>
-          <t>_res_.$AvgOfEmpties</t>
-        </is>
-      </c>
-      <c r="C36" s="5" t="inlineStr">
-        <is>
-          <t>avg(new Integer[] {null, null})</t>
-        </is>
-      </c>
-      <c r="D36" s="10" t="n"/>
-    </row>
-    <row r="37">
-      <c r="B37" s="9" t="inlineStr">
-        <is>
-          <t>_res_.$AvgOfNothing</t>
-        </is>
-      </c>
-      <c r="C37" s="5" t="inlineStr">
-        <is>
-          <t>avg(new int[] {})</t>
-        </is>
-      </c>
-      <c r="D37" s="10" t="n"/>
+      <c r="C37" s="8" t="n"/>
+      <c r="D37" s="4" t="n"/>
     </row>
     <row r="38">
       <c r="B38" s="9" t="inlineStr">
         <is>
-          <t>_res_.$AvgWithZeros</t>
+          <t>_res_.$AvgWithEmpty</t>
         </is>
       </c>
       <c r="C38" s="5" t="inlineStr">
         <is>
-          <t>avg(new int[] {1, 2, 0, 0, 6})</t>
+          <t>avg(5, null)</t>
         </is>
       </c>
       <c r="D38" s="10" t="n">
-        <v>1.8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="39">
       <c r="B39" s="9" t="inlineStr">
         <is>
-          <t>_res_.$AvgSkipsEmpties (6)</t>
+          <t>_res_.$AvgOfEmpties</t>
         </is>
       </c>
       <c r="C39" s="5" t="inlineStr">
         <is>
-          <t>avg(new Integer[] {-10, 5, null, null, 1})</t>
-        </is>
-      </c>
-      <c r="D39" s="10" t="n">
-        <v>-1.333333</v>
-      </c>
+          <t>avg(new Integer[] {null, null})</t>
+        </is>
+      </c>
+      <c r="D39" s="10" t="n"/>
     </row>
     <row r="40">
       <c r="B40" s="9" t="inlineStr">
         <is>
-          <t>_res_.$SumWithEmpty</t>
+          <t>_res_.$AvgOfNothing</t>
         </is>
       </c>
       <c r="C40" s="5" t="inlineStr">
         <is>
-          <t>Integer v = null; sum(5, v)</t>
-        </is>
-      </c>
-      <c r="D40" s="10" t="n">
-        <v>5</v>
-      </c>
+          <t>avg(new int[] {})</t>
+        </is>
+      </c>
+      <c r="D40" s="10" t="n"/>
     </row>
     <row r="41">
       <c r="B41" s="9" t="inlineStr">
         <is>
-          <t>_res_.$SumOfEmpties</t>
+          <t>_res_.$AvgWithZeros</t>
         </is>
       </c>
       <c r="C41" s="5" t="inlineStr">
         <is>
-          <t>sum(new Integer[] {null, null})</t>
-        </is>
-      </c>
-      <c r="D41" s="10" t="n"/>
+          <t>avg(new int[] {1, 2, 0, 0, 6})</t>
+        </is>
+      </c>
+      <c r="D41" s="10" t="n">
+        <v>1.8</v>
+      </c>
     </row>
     <row r="42">
       <c r="B42" s="9" t="inlineStr">
         <is>
-          <t>_res_.$ProductSkipsEmpties</t>
+          <t>_res_.$AvgSkipsEmpties (6)</t>
         </is>
       </c>
       <c r="C42" s="5" t="inlineStr">
         <is>
-          <t>product(new Integer[] {1, 2, null, null, 6})</t>
+          <t>avg(new Integer[] {-10, 5, null, null, 1})</t>
         </is>
       </c>
       <c r="D42" s="10" t="n">
-        <v>12</v>
+        <v>-1.333333</v>
       </c>
     </row>
     <row r="43">
       <c r="B43" s="9" t="inlineStr">
         <is>
-          <t>_res_.$ProductWithZeros</t>
+          <t>_res_.$SumWithEmpty</t>
         </is>
       </c>
       <c r="C43" s="5" t="inlineStr">
         <is>
-          <t>product(new int[] {1, 2, 0, 0, 6})</t>
+          <t>Integer v = null; sum(5, v)</t>
         </is>
       </c>
       <c r="D43" s="10" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="44">
       <c r="B44" s="9" t="inlineStr">
         <is>
-          <t>_res_.$ProductOfOne</t>
+          <t>_res_.$SumOfEmpties</t>
         </is>
       </c>
       <c r="C44" s="5" t="inlineStr">
         <is>
-          <t>product(new Integer[] {7})</t>
-        </is>
-      </c>
-      <c r="D44" s="10" t="n">
-        <v>7</v>
-      </c>
+          <t>sum(new Integer[] {null, null})</t>
+        </is>
+      </c>
+      <c r="D44" s="10" t="n"/>
     </row>
     <row r="45">
       <c r="B45" s="9" t="inlineStr">
         <is>
-          <t>_res_.$ProductOfNothing</t>
+          <t>_res_.$ProductSkipsEmpties</t>
         </is>
       </c>
       <c r="C45" s="5" t="inlineStr">
         <is>
-          <t>product(new Integer[] {})</t>
-        </is>
-      </c>
-      <c r="D45" s="10" t="n"/>
+          <t>product(new Integer[] {1, 2, null, null, 6})</t>
+        </is>
+      </c>
+      <c r="D45" s="10" t="n">
+        <v>12</v>
+      </c>
     </row>
     <row r="46">
       <c r="B46" s="9" t="inlineStr">
         <is>
-          <t>_res_.$ProductWithEmpty</t>
+          <t>_res_.$ProductWithZeros</t>
         </is>
       </c>
       <c r="C46" s="5" t="inlineStr">
         <is>
-          <t>Integer v = null; product(5, v)</t>
+          <t>product(new int[] {1, 2, 0, 0, 6})</t>
         </is>
       </c>
       <c r="D46" s="10" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="47">
       <c r="B47" s="9" t="inlineStr">
         <is>
-          <t>_res_.$MinWithZeros</t>
+          <t>_res_.$ProductOfOne</t>
         </is>
       </c>
       <c r="C47" s="5" t="inlineStr">
         <is>
-          <t>min(new int[] {1, 2, 0, 0, 6})</t>
+          <t>product(new Integer[] {7})</t>
         </is>
       </c>
       <c r="D47" s="10" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
     </row>
     <row r="48">
       <c r="B48" s="9" t="inlineStr">
         <is>
-          <t>_res_.$MinWithEmpty</t>
+          <t>_res_.$ProductOfNothing</t>
         </is>
       </c>
       <c r="C48" s="5" t="inlineStr">
         <is>
-          <t>Integer v = null; min(5, v)</t>
-        </is>
-      </c>
-      <c r="D48" s="10" t="n">
-        <v>5</v>
-      </c>
+          <t>product(new Integer[] {})</t>
+        </is>
+      </c>
+      <c r="D48" s="10" t="n"/>
     </row>
     <row r="49">
       <c r="B49" s="9" t="inlineStr">
         <is>
-          <t>_res_.$MaxWithEmpty</t>
+          <t>_res_.$ProductWithEmpty</t>
         </is>
       </c>
       <c r="C49" s="5" t="inlineStr">
         <is>
-          <t>Integer v = null; max(v, 1)</t>
+          <t>Integer v = null; product(5, v)</t>
         </is>
       </c>
       <c r="D49" s="10" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="50">
       <c r="B50" s="9" t="inlineStr">
         <is>
-          <t>_res_.$MinOfNothing</t>
+          <t>_res_.$MinWithZeros</t>
         </is>
       </c>
       <c r="C50" s="5" t="inlineStr">
         <is>
-          <t>min(new Integer[] {})</t>
-        </is>
-      </c>
-      <c r="D50" s="10" t="n"/>
+          <t>min(new int[] {1, 2, 0, 0, 6})</t>
+        </is>
+      </c>
+      <c r="D50" s="10" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="51">
       <c r="B51" s="9" t="inlineStr">
         <is>
-          <t>_res_.$MinWithNaN</t>
+          <t>_res_.$MinWithEmpty</t>
         </is>
       </c>
       <c r="C51" s="5" t="inlineStr">
         <is>
-          <t>min(Double.NaN, 1.5)</t>
-        </is>
-      </c>
-      <c r="D51" s="10" t="inlineStr">
-        <is>
-          <t>NaN</t>
-        </is>
+          <t>Integer v = null; min(5, v)</t>
+        </is>
+      </c>
+      <c r="D51" s="10" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="52">
       <c r="B52" s="9" t="inlineStr">
         <is>
-          <t>_res_.$MaxWithNaN</t>
+          <t>_res_.$MaxWithEmpty</t>
         </is>
       </c>
       <c r="C52" s="5" t="inlineStr">
         <is>
-          <t>max(1.5, Double.NaN)</t>
-        </is>
-      </c>
-      <c r="D52" s="10" t="inlineStr">
-        <is>
-          <t>NaN</t>
-        </is>
+          <t>Integer v = null; max(v, 1)</t>
+        </is>
+      </c>
+      <c r="D52" s="10" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="53">
       <c r="B53" s="9" t="inlineStr">
         <is>
-          <t>_res_.$MinOfArrayWithNaN</t>
+          <t>_res_.$MinOfNothing</t>
         </is>
       </c>
       <c r="C53" s="5" t="inlineStr">
         <is>
-          <t>min(new Double[] {3, null, Double.NaN, 1})</t>
-        </is>
-      </c>
-      <c r="D53" s="10" t="inlineStr">
-        <is>
-          <t>NaN</t>
-        </is>
-      </c>
+          <t>min(new Integer[] {})</t>
+        </is>
+      </c>
+      <c r="D53" s="10" t="n"/>
     </row>
     <row r="54">
       <c r="B54" s="9" t="inlineStr">
         <is>
-          <t>_res_.$MaxOfArrayWithNaN</t>
+          <t>_res_.$MinWithNaN</t>
         </is>
       </c>
       <c r="C54" s="5" t="inlineStr">
         <is>
-          <t>max(new double[] {Double.NaN, 3, 1})</t>
+          <t>min(Double.NaN, 1.5)</t>
         </is>
       </c>
       <c r="D54" s="10" t="inlineStr">
@@ -1886,642 +1871,744 @@
     <row r="55">
       <c r="B55" s="9" t="inlineStr">
         <is>
-          <t>_res_.$MedianWithZeros</t>
+          <t>_res_.$MaxWithNaN</t>
         </is>
       </c>
       <c r="C55" s="5" t="inlineStr">
         <is>
-          <t>median(new int[] {1, 2, 0, 0, 6})</t>
-        </is>
-      </c>
-      <c r="D55" s="10" t="n">
-        <v>1</v>
+          <t>max(1.5, Double.NaN)</t>
+        </is>
+      </c>
+      <c r="D55" s="10" t="inlineStr">
+        <is>
+          <t>NaN</t>
+        </is>
       </c>
     </row>
     <row r="56">
       <c r="B56" s="9" t="inlineStr">
         <is>
-          <t>_res_.$MedianSkipsEmpties</t>
+          <t>_res_.$MinOfArrayWithNaN</t>
         </is>
       </c>
       <c r="C56" s="5" t="inlineStr">
         <is>
-          <t>median(new Integer[] {1, 2, null, null, 6})</t>
-        </is>
-      </c>
-      <c r="D56" s="10" t="n">
-        <v>2</v>
+          <t>min(new Double[] {3, null, Double.NaN, 1})</t>
+        </is>
+      </c>
+      <c r="D56" s="10" t="inlineStr">
+        <is>
+          <t>NaN</t>
+        </is>
       </c>
     </row>
     <row r="57">
       <c r="B57" s="9" t="inlineStr">
         <is>
-          <t>_res_.$MedianOfNothing</t>
+          <t>_res_.$MaxOfArrayWithNaN</t>
         </is>
       </c>
       <c r="C57" s="5" t="inlineStr">
         <is>
-          <t>median(new Integer[] {null})</t>
-        </is>
-      </c>
-      <c r="D57" s="10" t="n"/>
+          <t>max(new double[] {Double.NaN, 3, 1})</t>
+        </is>
+      </c>
+      <c r="D57" s="10" t="inlineStr">
+        <is>
+          <t>NaN</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="B58" s="9" t="inlineStr">
         <is>
-          <t>_res_.$SmallSkipsEmpties</t>
+          <t>_res_.$MedianWithZeros</t>
         </is>
       </c>
       <c r="C58" s="5" t="inlineStr">
         <is>
-          <t>small(new Integer[] {1, 2, null, null, 6}, 3)</t>
+          <t>median(new int[] {1, 2, 0, 0, 6})</t>
         </is>
       </c>
       <c r="D58" s="10" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
     </row>
     <row r="59">
       <c r="B59" s="9" t="inlineStr">
         <is>
+          <t>_res_.$MedianSkipsEmpties</t>
+        </is>
+      </c>
+      <c r="C59" s="5" t="inlineStr">
+        <is>
+          <t>median(new Integer[] {1, 2, null, null, 6})</t>
+        </is>
+      </c>
+      <c r="D59" s="10" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="B60" s="9" t="inlineStr">
+        <is>
+          <t>_res_.$MedianOfNothing</t>
+        </is>
+      </c>
+      <c r="C60" s="5" t="inlineStr">
+        <is>
+          <t>median(new Integer[] {null})</t>
+        </is>
+      </c>
+      <c r="D60" s="10" t="n"/>
+    </row>
+    <row r="61">
+      <c r="B61" s="9" t="inlineStr">
+        <is>
+          <t>_res_.$MedianWithNaN</t>
+        </is>
+      </c>
+      <c r="C61" s="5" t="inlineStr">
+        <is>
+          <t>median(new Double[] {3, Double.NaN, 1})</t>
+        </is>
+      </c>
+      <c r="D61" s="10" t="inlineStr">
+        <is>
+          <t>NaN</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="B62" s="9" t="inlineStr">
+        <is>
+          <t>_res_.$SmallSkipsEmpties</t>
+        </is>
+      </c>
+      <c r="C62" s="5" t="inlineStr">
+        <is>
+          <t>small(new Integer[] {1, 2, null, null, 6}, 3)</t>
+        </is>
+      </c>
+      <c r="D62" s="10" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="B63" s="9" t="inlineStr">
+        <is>
           <t>_res_.$SmallWithZeros</t>
         </is>
       </c>
-      <c r="C59" s="5" t="inlineStr">
+      <c r="C63" s="5" t="inlineStr">
         <is>
           <t>small(new int[] {1, 2, 0, 0, 6}, 3)</t>
         </is>
       </c>
-      <c r="D59" s="10" t="n">
+      <c r="D63" s="10" t="n">
         <v>1</v>
       </c>
     </row>
-    <row r="61" ht="43.5" customHeight="1">
-      <c r="B61" s="2" t="inlineStr">
+    <row r="64">
+      <c r="B64" s="9" t="inlineStr">
+        <is>
+          <t>_res_.$SmallWithNaN</t>
+        </is>
+      </c>
+      <c r="C64" s="5" t="inlineStr">
+        <is>
+          <t>small(new Double[] {3, Double.NaN, 1}, 1)</t>
+        </is>
+      </c>
+      <c r="D64" s="10" t="inlineStr">
+        <is>
+          <t>NaN</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="B65" s="9" t="inlineStr">
+        <is>
+          <t>_res_.$BigWithNaN</t>
+        </is>
+      </c>
+      <c r="C65" s="5" t="inlineStr">
+        <is>
+          <t>big(new double[] {3, Double.NaN, 1}, 2)</t>
+        </is>
+      </c>
+      <c r="D65" s="10" t="inlineStr">
+        <is>
+          <t>NaN</t>
+        </is>
+      </c>
+    </row>
+    <row r="67" ht="43.5" customHeight="1">
+      <c r="B67" s="2" t="inlineStr">
         <is>
           <t>sum, min and max keep the type of the elements, but the sum of Byte or Short values is an Integer, so it does not wrap around at 127. The sum of Integer values wraps around past 2147483647 like "+". product returns a Double, except for BigInteger and BigDecimal. avg and median return a Double, a Float for Float elements and a BigDecimal for BigInteger and BigDecimal elements. A two-dimensional array gives one sum per row.</t>
         </is>
       </c>
     </row>
-    <row r="63">
-      <c r="B63" s="3" t="inlineStr">
+    <row r="69">
+      <c r="B69" s="3" t="inlineStr">
         <is>
           <t>Spreadsheet SpreadsheetResult AggregateTypes()</t>
         </is>
       </c>
-      <c r="C63" s="4" t="n"/>
-    </row>
-    <row r="64">
-      <c r="B64" s="5" t="inlineStr">
+      <c r="C69" s="4" t="n"/>
+    </row>
+    <row r="70">
+      <c r="B70" s="5" t="inlineStr">
         <is>
           <t>Step</t>
         </is>
       </c>
-      <c r="C64" s="5" t="inlineStr">
+      <c r="C70" s="5" t="inlineStr">
         <is>
           <t>Value</t>
-        </is>
-      </c>
-    </row>
-    <row r="65">
-      <c r="B65" s="6" t="inlineStr">
-        <is>
-          <t>ByteSum</t>
-        </is>
-      </c>
-      <c r="C65" s="7" t="inlineStr">
-        <is>
-          <t>= sum((byte) 100, (byte) 100)</t>
-        </is>
-      </c>
-    </row>
-    <row r="66">
-      <c r="B66" s="6" t="inlineStr">
-        <is>
-          <t>ByteSumType</t>
-        </is>
-      </c>
-      <c r="C66" s="7" t="inlineStr">
-        <is>
-          <t>= sum((byte) 100, (byte) 100).getClass().getSimpleName()</t>
-        </is>
-      </c>
-    </row>
-    <row r="67">
-      <c r="B67" s="6" t="inlineStr">
-        <is>
-          <t>IntegerSumWraps</t>
-        </is>
-      </c>
-      <c r="C67" s="7" t="inlineStr">
-        <is>
-          <t>= sum(Integer.MAX_VALUE, 1)</t>
-        </is>
-      </c>
-    </row>
-    <row r="68">
-      <c r="B68" s="6" t="inlineStr">
-        <is>
-          <t>FloatSumType</t>
-        </is>
-      </c>
-      <c r="C68" s="7" t="inlineStr">
-        <is>
-          <t>= sum(new Float[] {1.5f, 2f}).getClass().getSimpleName()</t>
-        </is>
-      </c>
-    </row>
-    <row r="69">
-      <c r="B69" s="6" t="inlineStr">
-        <is>
-          <t>BigIntegerSum</t>
-        </is>
-      </c>
-      <c r="C69" s="7" t="inlineStr">
-        <is>
-          <t>= sum(new BigInteger[] {(BigInteger) 1, null})</t>
-        </is>
-      </c>
-    </row>
-    <row r="70">
-      <c r="B70" s="6" t="inlineStr">
-        <is>
-          <t>ByteProduct</t>
-        </is>
-      </c>
-      <c r="C70" s="7" t="inlineStr">
-        <is>
-          <t>= product((byte) -100, (byte) 100)</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="B71" s="6" t="inlineStr">
         <is>
-          <t>ProductType</t>
+          <t>ByteSum</t>
         </is>
       </c>
       <c r="C71" s="7" t="inlineStr">
         <is>
-          <t>= product(new Integer[] {3, 4}).getClass().getSimpleName()</t>
+          <t>= sum((byte) 100, (byte) 100)</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="B72" s="6" t="inlineStr">
         <is>
-          <t>FloatProductType</t>
+          <t>ByteSumType</t>
         </is>
       </c>
       <c r="C72" s="7" t="inlineStr">
         <is>
-          <t>= product(new Float[] {1.5f, 2f}).getClass().getSimpleName()</t>
+          <t>= sum((byte) 100, (byte) 100).getClass().getSimpleName()</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="B73" s="6" t="inlineStr">
         <is>
-          <t>BigIntegerProductType</t>
+          <t>IntegerSumWraps</t>
         </is>
       </c>
       <c r="C73" s="7" t="inlineStr">
         <is>
-          <t>= product(new BigInteger[] {(BigInteger) 3, (BigInteger) 4}).getClass().getSimpleName()</t>
+          <t>= sum(Integer.MAX_VALUE, 1)</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="B74" s="6" t="inlineStr">
         <is>
-          <t>ByteMaxType</t>
+          <t>FloatSumType</t>
         </is>
       </c>
       <c r="C74" s="7" t="inlineStr">
         <is>
-          <t>= max((byte) -100, (byte) 100).getClass().getSimpleName()</t>
+          <t>= sum(new Float[] {1.5f, 2f}).getClass().getSimpleName()</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="B75" s="6" t="inlineStr">
         <is>
-          <t>BigIntegerMax</t>
+          <t>BigIntegerSum</t>
         </is>
       </c>
       <c r="C75" s="7" t="inlineStr">
         <is>
-          <t>= max(new BigInteger[] {(BigInteger) 3, (BigInteger) 4})</t>
+          <t>= sum(new BigInteger[] {(BigInteger) 1, null})</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="B76" s="6" t="inlineStr">
         <is>
-          <t>LongAvgType</t>
+          <t>ByteProduct</t>
         </is>
       </c>
       <c r="C76" s="7" t="inlineStr">
         <is>
-          <t>= avg(new Long[] {1L, 2L}).getClass().getSimpleName()</t>
+          <t>= product((byte) -100, (byte) 100)</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="B77" s="6" t="inlineStr">
         <is>
-          <t>FloatAvgType</t>
+          <t>ProductType</t>
         </is>
       </c>
       <c r="C77" s="7" t="inlineStr">
         <is>
-          <t>= avg(new Float[] {1f, 2f}).getClass().getSimpleName()</t>
+          <t>= product(new Integer[] {3, 4}).getClass().getSimpleName()</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="B78" s="6" t="inlineStr">
         <is>
-          <t>BigIntegerAvg</t>
+          <t>FloatProductType</t>
         </is>
       </c>
       <c r="C78" s="7" t="inlineStr">
         <is>
-          <t>= avg(new BigInteger[] {(BigInteger) 1, (BigInteger) 2})</t>
+          <t>= product(new Float[] {1.5f, 2f}).getClass().getSimpleName()</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="B79" s="6" t="inlineStr">
         <is>
-          <t>BigIntegerAvgType</t>
+          <t>BigIntegerProductType</t>
         </is>
       </c>
       <c r="C79" s="7" t="inlineStr">
         <is>
-          <t>= avg(new BigInteger[] {(BigInteger) 1, (BigInteger) 2}).getClass().getSimpleName()</t>
+          <t>= product(new BigInteger[] {(BigInteger) 3, (BigInteger) 4}).getClass().getSimpleName()</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="B80" s="6" t="inlineStr">
         <is>
-          <t>FloatMedianType</t>
+          <t>ByteMaxType</t>
         </is>
       </c>
       <c r="C80" s="7" t="inlineStr">
         <is>
-          <t>= median(new Float[] {1f, 2f}).getClass().getSimpleName()</t>
+          <t>= max((byte) -100, (byte) 100).getClass().getSimpleName()</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="B81" s="6" t="inlineStr">
         <is>
-          <t>DecimalMedian</t>
+          <t>BigIntegerMax</t>
         </is>
       </c>
       <c r="C81" s="7" t="inlineStr">
         <is>
-          <t>= median(new BigDecimal[] {(BigDecimal) 1, (BigDecimal) 2})</t>
+          <t>= max(new BigInteger[] {(BigInteger) 3, (BigInteger) 4})</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="B82" s="6" t="inlineStr">
         <is>
-          <t>LongMedian</t>
+          <t>LongAvgType</t>
         </is>
       </c>
       <c r="C82" s="7" t="inlineStr">
         <is>
-          <t>= median(new Long[] {1L, 2L, 3L, 4L})</t>
+          <t>= avg(new Long[] {1L, 2L}).getClass().getSimpleName()</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="B83" s="6" t="inlineStr">
         <is>
+          <t>FloatAvgType</t>
+        </is>
+      </c>
+      <c r="C83" s="7" t="inlineStr">
+        <is>
+          <t>= avg(new Float[] {1f, 2f}).getClass().getSimpleName()</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="B84" s="6" t="inlineStr">
+        <is>
+          <t>BigIntegerAvg</t>
+        </is>
+      </c>
+      <c r="C84" s="7" t="inlineStr">
+        <is>
+          <t>= avg(new BigInteger[] {(BigInteger) 1, (BigInteger) 2})</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="B85" s="6" t="inlineStr">
+        <is>
+          <t>BigIntegerAvgType</t>
+        </is>
+      </c>
+      <c r="C85" s="7" t="inlineStr">
+        <is>
+          <t>= avg(new BigInteger[] {(BigInteger) 1, (BigInteger) 2}).getClass().getSimpleName()</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="B86" s="6" t="inlineStr">
+        <is>
+          <t>FloatMedianType</t>
+        </is>
+      </c>
+      <c r="C86" s="7" t="inlineStr">
+        <is>
+          <t>= median(new Float[] {1f, 2f}).getClass().getSimpleName()</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="B87" s="6" t="inlineStr">
+        <is>
+          <t>DecimalMedian</t>
+        </is>
+      </c>
+      <c r="C87" s="7" t="inlineStr">
+        <is>
+          <t>= median(new BigDecimal[] {(BigDecimal) 1, (BigDecimal) 2})</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="B88" s="6" t="inlineStr">
+        <is>
+          <t>LongMedian</t>
+        </is>
+      </c>
+      <c r="C88" s="7" t="inlineStr">
+        <is>
+          <t>= median(new Long[] {1L, 2L, 3L, 4L})</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="B89" s="6" t="inlineStr">
+        <is>
           <t>SumOfRows</t>
         </is>
       </c>
-      <c r="C83" s="7" t="inlineStr">
+      <c r="C89" s="7" t="inlineStr">
         <is>
           <t>= sum(new Integer[][] {{1, 2}, {3}})</t>
         </is>
       </c>
     </row>
-    <row r="85">
-      <c r="B85" s="3" t="inlineStr">
+    <row r="91">
+      <c r="B91" s="3" t="inlineStr">
         <is>
           <t>Test AggregateTypes AggregateTypesTest</t>
         </is>
       </c>
-      <c r="C85" s="8" t="n"/>
-      <c r="D85" s="4" t="n"/>
-    </row>
-    <row r="86">
-      <c r="B86" s="9" t="inlineStr">
-        <is>
-          <t>_res_.$ByteSum</t>
-        </is>
-      </c>
-      <c r="C86" s="5" t="inlineStr">
-        <is>
-          <t>sum((byte) 100, (byte) 100)</t>
-        </is>
-      </c>
-      <c r="D86" s="10" t="n">
-        <v>200</v>
-      </c>
-    </row>
-    <row r="87">
-      <c r="B87" s="9" t="inlineStr">
-        <is>
-          <t>_res_.$ByteSumType</t>
-        </is>
-      </c>
-      <c r="C87" s="5" t="inlineStr">
-        <is>
-          <t>sum((byte) 100, (byte) 100).getClass().getSimpleName()</t>
-        </is>
-      </c>
-      <c r="D87" s="10" t="inlineStr">
-        <is>
-          <t>Integer</t>
-        </is>
-      </c>
-    </row>
-    <row r="88">
-      <c r="B88" s="9" t="inlineStr">
-        <is>
-          <t>_res_.$IntegerSumWraps</t>
-        </is>
-      </c>
-      <c r="C88" s="5" t="inlineStr">
-        <is>
-          <t>sum(Integer.MAX_VALUE, 1)</t>
-        </is>
-      </c>
-      <c r="D88" s="10" t="n">
-        <v>-2147483648</v>
-      </c>
-    </row>
-    <row r="89">
-      <c r="B89" s="9" t="inlineStr">
-        <is>
-          <t>_res_.$FloatSumType</t>
-        </is>
-      </c>
-      <c r="C89" s="5" t="inlineStr">
-        <is>
-          <t>sum(new Float[] {1.5f, 2f}).getClass().getSimpleName()</t>
-        </is>
-      </c>
-      <c r="D89" s="10" t="inlineStr">
-        <is>
-          <t>Float</t>
-        </is>
-      </c>
-    </row>
-    <row r="90">
-      <c r="B90" s="9" t="inlineStr">
-        <is>
-          <t>_res_.$BigIntegerSum</t>
-        </is>
-      </c>
-      <c r="C90" s="5" t="inlineStr">
-        <is>
-          <t>sum(new BigInteger[] {(BigInteger) 1, null})</t>
-        </is>
-      </c>
-      <c r="D90" s="10" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="91">
-      <c r="B91" s="9" t="inlineStr">
-        <is>
-          <t>_res_.$ByteProduct</t>
-        </is>
-      </c>
-      <c r="C91" s="5" t="inlineStr">
-        <is>
-          <t>product((byte) -100, (byte) 100)</t>
-        </is>
-      </c>
-      <c r="D91" s="10" t="n">
-        <v>-10000</v>
-      </c>
+      <c r="C91" s="8" t="n"/>
+      <c r="D91" s="4" t="n"/>
     </row>
     <row r="92">
       <c r="B92" s="9" t="inlineStr">
         <is>
-          <t>_res_.$ProductType</t>
+          <t>_res_.$ByteSum</t>
         </is>
       </c>
       <c r="C92" s="5" t="inlineStr">
         <is>
-          <t>product(new Integer[] {3, 4}).getClass().getSimpleName()</t>
-        </is>
-      </c>
-      <c r="D92" s="10" t="inlineStr">
-        <is>
-          <t>Double</t>
-        </is>
+          <t>sum((byte) 100, (byte) 100)</t>
+        </is>
+      </c>
+      <c r="D92" s="10" t="n">
+        <v>200</v>
       </c>
     </row>
     <row r="93">
       <c r="B93" s="9" t="inlineStr">
         <is>
-          <t>_res_.$FloatProductType</t>
+          <t>_res_.$ByteSumType</t>
         </is>
       </c>
       <c r="C93" s="5" t="inlineStr">
         <is>
-          <t>product(new Float[] {1.5f, 2f}).getClass().getSimpleName()</t>
+          <t>sum((byte) 100, (byte) 100).getClass().getSimpleName()</t>
         </is>
       </c>
       <c r="D93" s="10" t="inlineStr">
         <is>
-          <t>Double</t>
+          <t>Integer</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="B94" s="9" t="inlineStr">
         <is>
-          <t>_res_.$BigIntegerProductType</t>
+          <t>_res_.$IntegerSumWraps</t>
         </is>
       </c>
       <c r="C94" s="5" t="inlineStr">
         <is>
-          <t>product(new BigInteger[] {(BigInteger) 3, (BigInteger) 4}).getClass().getSimpleName()</t>
-        </is>
-      </c>
-      <c r="D94" s="10" t="inlineStr">
-        <is>
-          <t>BigInteger</t>
-        </is>
+          <t>sum(Integer.MAX_VALUE, 1)</t>
+        </is>
+      </c>
+      <c r="D94" s="10" t="n">
+        <v>-2147483648</v>
       </c>
     </row>
     <row r="95">
       <c r="B95" s="9" t="inlineStr">
         <is>
-          <t>_res_.$ByteMaxType</t>
+          <t>_res_.$FloatSumType</t>
         </is>
       </c>
       <c r="C95" s="5" t="inlineStr">
         <is>
-          <t>max((byte) -100, (byte) 100).getClass().getSimpleName()</t>
+          <t>sum(new Float[] {1.5f, 2f}).getClass().getSimpleName()</t>
         </is>
       </c>
       <c r="D95" s="10" t="inlineStr">
         <is>
-          <t>Byte</t>
+          <t>Float</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="B96" s="9" t="inlineStr">
         <is>
-          <t>_res_.$BigIntegerMax</t>
+          <t>_res_.$BigIntegerSum</t>
         </is>
       </c>
       <c r="C96" s="5" t="inlineStr">
         <is>
-          <t>max(new BigInteger[] {(BigInteger) 3, (BigInteger) 4})</t>
+          <t>sum(new BigInteger[] {(BigInteger) 1, null})</t>
         </is>
       </c>
       <c r="D96" s="10" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="97">
       <c r="B97" s="9" t="inlineStr">
         <is>
-          <t>_res_.$LongAvgType</t>
+          <t>_res_.$ByteProduct</t>
         </is>
       </c>
       <c r="C97" s="5" t="inlineStr">
         <is>
-          <t>avg(new Long[] {1L, 2L}).getClass().getSimpleName()</t>
-        </is>
-      </c>
-      <c r="D97" s="10" t="inlineStr">
-        <is>
-          <t>Double</t>
-        </is>
+          <t>product((byte) -100, (byte) 100)</t>
+        </is>
+      </c>
+      <c r="D97" s="10" t="n">
+        <v>-10000</v>
       </c>
     </row>
     <row r="98">
       <c r="B98" s="9" t="inlineStr">
         <is>
-          <t>_res_.$FloatAvgType</t>
+          <t>_res_.$ProductType</t>
         </is>
       </c>
       <c r="C98" s="5" t="inlineStr">
         <is>
-          <t>avg(new Float[] {1f, 2f}).getClass().getSimpleName()</t>
+          <t>product(new Integer[] {3, 4}).getClass().getSimpleName()</t>
         </is>
       </c>
       <c r="D98" s="10" t="inlineStr">
         <is>
-          <t>Float</t>
+          <t>Double</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="B99" s="9" t="inlineStr">
         <is>
-          <t>_res_.$BigIntegerAvg</t>
+          <t>_res_.$FloatProductType</t>
         </is>
       </c>
       <c r="C99" s="5" t="inlineStr">
         <is>
-          <t>avg(new BigInteger[] {(BigInteger) 1, (BigInteger) 2})</t>
-        </is>
-      </c>
-      <c r="D99" s="10" t="n">
-        <v>1.5</v>
+          <t>product(new Float[] {1.5f, 2f}).getClass().getSimpleName()</t>
+        </is>
+      </c>
+      <c r="D99" s="10" t="inlineStr">
+        <is>
+          <t>Double</t>
+        </is>
       </c>
     </row>
     <row r="100">
       <c r="B100" s="9" t="inlineStr">
         <is>
-          <t>_res_.$BigIntegerAvgType</t>
+          <t>_res_.$BigIntegerProductType</t>
         </is>
       </c>
       <c r="C100" s="5" t="inlineStr">
         <is>
-          <t>avg(new BigInteger[] {(BigInteger) 1, (BigInteger) 2}).getClass().getSimpleName()</t>
+          <t>product(new BigInteger[] {(BigInteger) 3, (BigInteger) 4}).getClass().getSimpleName()</t>
         </is>
       </c>
       <c r="D100" s="10" t="inlineStr">
         <is>
-          <t>BigDecimal</t>
+          <t>BigInteger</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="B101" s="9" t="inlineStr">
         <is>
-          <t>_res_.$FloatMedianType</t>
+          <t>_res_.$ByteMaxType</t>
         </is>
       </c>
       <c r="C101" s="5" t="inlineStr">
         <is>
-          <t>median(new Float[] {1f, 2f}).getClass().getSimpleName()</t>
+          <t>max((byte) -100, (byte) 100).getClass().getSimpleName()</t>
         </is>
       </c>
       <c r="D101" s="10" t="inlineStr">
         <is>
-          <t>Float</t>
+          <t>Byte</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="B102" s="9" t="inlineStr">
         <is>
-          <t>_res_.$DecimalMedian</t>
+          <t>_res_.$BigIntegerMax</t>
         </is>
       </c>
       <c r="C102" s="5" t="inlineStr">
         <is>
-          <t>median(new BigDecimal[] {(BigDecimal) 1, (BigDecimal) 2})</t>
+          <t>max(new BigInteger[] {(BigInteger) 3, (BigInteger) 4})</t>
         </is>
       </c>
       <c r="D102" s="10" t="n">
-        <v>1.5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="103">
       <c r="B103" s="9" t="inlineStr">
         <is>
-          <t>_res_.$LongMedian</t>
+          <t>_res_.$LongAvgType</t>
         </is>
       </c>
       <c r="C103" s="5" t="inlineStr">
         <is>
-          <t>median(new Long[] {1L, 2L, 3L, 4L})</t>
-        </is>
-      </c>
-      <c r="D103" s="10" t="n">
-        <v>2.5</v>
+          <t>avg(new Long[] {1L, 2L}).getClass().getSimpleName()</t>
+        </is>
+      </c>
+      <c r="D103" s="10" t="inlineStr">
+        <is>
+          <t>Double</t>
+        </is>
       </c>
     </row>
     <row r="104">
       <c r="B104" s="9" t="inlineStr">
         <is>
+          <t>_res_.$FloatAvgType</t>
+        </is>
+      </c>
+      <c r="C104" s="5" t="inlineStr">
+        <is>
+          <t>avg(new Float[] {1f, 2f}).getClass().getSimpleName()</t>
+        </is>
+      </c>
+      <c r="D104" s="10" t="inlineStr">
+        <is>
+          <t>Float</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="B105" s="9" t="inlineStr">
+        <is>
+          <t>_res_.$BigIntegerAvg</t>
+        </is>
+      </c>
+      <c r="C105" s="5" t="inlineStr">
+        <is>
+          <t>avg(new BigInteger[] {(BigInteger) 1, (BigInteger) 2})</t>
+        </is>
+      </c>
+      <c r="D105" s="10" t="n">
+        <v>1.5</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="B106" s="9" t="inlineStr">
+        <is>
+          <t>_res_.$BigIntegerAvgType</t>
+        </is>
+      </c>
+      <c r="C106" s="5" t="inlineStr">
+        <is>
+          <t>avg(new BigInteger[] {(BigInteger) 1, (BigInteger) 2}).getClass().getSimpleName()</t>
+        </is>
+      </c>
+      <c r="D106" s="10" t="inlineStr">
+        <is>
+          <t>BigDecimal</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="B107" s="9" t="inlineStr">
+        <is>
+          <t>_res_.$FloatMedianType</t>
+        </is>
+      </c>
+      <c r="C107" s="5" t="inlineStr">
+        <is>
+          <t>median(new Float[] {1f, 2f}).getClass().getSimpleName()</t>
+        </is>
+      </c>
+      <c r="D107" s="10" t="inlineStr">
+        <is>
+          <t>Float</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="B108" s="9" t="inlineStr">
+        <is>
+          <t>_res_.$DecimalMedian</t>
+        </is>
+      </c>
+      <c r="C108" s="5" t="inlineStr">
+        <is>
+          <t>median(new BigDecimal[] {(BigDecimal) 1, (BigDecimal) 2})</t>
+        </is>
+      </c>
+      <c r="D108" s="10" t="n">
+        <v>1.5</v>
+      </c>
+    </row>
+    <row r="109">
+      <c r="B109" s="9" t="inlineStr">
+        <is>
+          <t>_res_.$LongMedian</t>
+        </is>
+      </c>
+      <c r="C109" s="5" t="inlineStr">
+        <is>
+          <t>median(new Long[] {1L, 2L, 3L, 4L})</t>
+        </is>
+      </c>
+      <c r="D109" s="10" t="n">
+        <v>2.5</v>
+      </c>
+    </row>
+    <row r="110">
+      <c r="B110" s="9" t="inlineStr">
+        <is>
           <t>_res_.$SumOfRows</t>
         </is>
       </c>
-      <c r="C104" s="5" t="inlineStr">
+      <c r="C110" s="5" t="inlineStr">
         <is>
           <t>sum(new Integer[][] {{1, 2}, {3}})</t>
         </is>
       </c>
-      <c r="D104" s="10" t="inlineStr">
+      <c r="D110" s="10" t="inlineStr">
         <is>
           <t>3, 3</t>
         </is>
@@ -2529,11 +2616,11 @@
     </row>
   </sheetData>
   <mergeCells count="6">
-    <mergeCell ref="B63:C63"/>
+    <mergeCell ref="B69:C69"/>
     <mergeCell ref="B6:C6"/>
-    <mergeCell ref="B61:I61"/>
-    <mergeCell ref="B34:D34"/>
-    <mergeCell ref="B85:D85"/>
+    <mergeCell ref="B67:I67"/>
+    <mergeCell ref="B37:D37"/>
+    <mergeCell ref="B91:D91"/>
     <mergeCell ref="B4:I4"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
EPBDS-7001 Round sum, avg and product of Doubles once with Kahan compensation
</commit_message>
<xml_diff>
--- a/DEV/org.openl.rules.demo/src/org.openl.rules.demo.examples/Example-4-Reference-Guide/rules/7-Functions/AggregateFunctions.xlsx
+++ b/DEV/org.openl.rules.demo/src/org.openl.rules.demo.examples/Example-4-Reference-Guide/rules/7-Functions/AggregateFunctions.xlsx
@@ -10,9 +10,25 @@
     <sheet name="Aggregates" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="EmptyAndTypes" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
-  <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
+</file>
+
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
+  <si>
+    <t>sum, avg, product, min, max and median take an array or a list of values. Empty elements are skipped. min and max also compare dates and texts. The result of sum and product keeps the type of the elements; avg and median return a fraction. Fractions are added as the decimals they show and rounded once, so ten times 0.1 sum to exactly 1.</t>
+  </si>
+  <si>
+    <t>= sum(new Double[] {0.1, 0.1, 0.1, 0.1, 0.1, 0.1, 0.1, 0.1, 0.1, 0.1}) ==== 1.0</t>
+  </si>
+  <si>
+    <t>sum(new Double[] {0.1, 0.1, 0.1, 0.1, 0.1, 0.1, 0.1, 0.1, 0.1, 0.1}) ==== 1.0</t>
+  </si>
+  <si>
+    <t>true</t>
+  </si>
+</sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
@@ -548,13 +564,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B2:I60"/>
+  <dimension ref="B2:D60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="2.5" customWidth="1" min="1" max="1"/>
-    <col width="27.2" customWidth="1" min="2" max="2"/>
-    <col width="68.2" customWidth="1" min="3" max="3"/>
-    <col width="12.5" customWidth="1" min="4" max="4"/>
+    <col min="1" max="1" customWidth="true" width="2.5"/>
+    <col min="2" max="2" customWidth="true" width="27.2"/>
+    <col min="3" max="3" customWidth="true" width="68.2"/>
+    <col min="4" max="4" customWidth="true" width="12.5"/>
   </cols>
   <sheetData>
     <row r="2">
@@ -565,10 +581,8 @@
       </c>
     </row>
     <row r="4" ht="30" customHeight="1">
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>sum, avg, product, min, max and median take an array or a list of values. Empty elements are skipped. min and max also compare dates and texts. The result of sum and product keeps the type of the elements; avg and median return a fraction.</t>
-        </is>
+      <c r="B4" s="2" t="s">
+        <v>0</v>
       </c>
     </row>
     <row r="6">
@@ -645,10 +659,8 @@
           <t>SumDecimals</t>
         </is>
       </c>
-      <c r="C12" s="7" t="inlineStr">
-        <is>
-          <t>= sum(new BigDecimal[] {(BigDecimal) 0.1, (BigDecimal) 0.2})</t>
-        </is>
+      <c r="C12" s="7" t="s">
+        <v>1</v>
       </c>
     </row>
     <row r="13">
@@ -832,13 +844,11 @@
           <t>_res_.$SumDecimals</t>
         </is>
       </c>
-      <c r="C28" s="5" t="inlineStr">
-        <is>
-          <t>sum(new BigDecimal[] {(BigDecimal) 0.1, (BigDecimal) 0.2})</t>
-        </is>
-      </c>
-      <c r="D28" s="10" t="n">
-        <v>0.3</v>
+      <c r="C28" s="5" t="s">
+        <v>2</v>
+      </c>
+      <c r="D28" s="10" t="s">
+        <v>3</v>
       </c>
     </row>
     <row r="29">
@@ -1233,13 +1243,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B2:I110"/>
+  <dimension ref="B2:D110"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="2.5" customWidth="1" min="1" max="1"/>
-    <col width="31.4" customWidth="1" min="2" max="2"/>
-    <col width="70" customWidth="1" min="3" max="3"/>
-    <col width="13.6" customWidth="1" min="4" max="4"/>
+    <col min="1" max="1" customWidth="true" width="2.5"/>
+    <col min="2" max="2" customWidth="true" width="31.4"/>
+    <col min="3" max="3" customWidth="true" width="70.0"/>
+    <col min="4" max="4" customWidth="true" width="13.6"/>
   </cols>
   <sheetData>
     <row r="2">

</xml_diff>